<commit_message>
docs(datos): el seguimiento GPS llega como link por unidad, no por API
</commit_message>
<xml_diff>
--- a/docs/captura-datos/DemoLogistics_plantilla_datos.xlsx
+++ b/docs/captura-datos/DemoLogistics_plantilla_datos.xlsx
@@ -382,6 +382,16 @@
         <t>Tipo de cobertura y montos relevantes</t>
       </text>
     </comment>
+    <comment ref="Y2" authorId="0" shapeId="0">
+      <text>
+        <t>Pegue el link con el que se rastrea esta unidad. Si es el mismo para toda la flota, déjelo sólo en la primera fila y anótelo en Notas</t>
+      </text>
+    </comment>
+    <comment ref="Z2" authorId="0" shapeId="0">
+      <text>
+        <t>Aclaraciones sobre la unidad, su documentación o su seguimiento</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -715,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:C35"/>
+  <dimension ref="B2:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -862,75 +872,75 @@
     <row r="24">
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Telemetría / GPS</t>
+          <t>Seguimiento GPS</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Si cuentan con un proveedor de rastreo satelital, necesitamos saber:</t>
+          <t>El rastreo se consulta con un link por unidad. Sólo hay que pegarlo en la plantilla:</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>•  Proveedor (Samsara, Motive, Wialon, Geotab, u otro).</t>
+          <t>•  En la hoja «1. Unidades», columna «Link de seguimiento (GPS)», pegue el link de cada unidad.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>•  Si ofrece API o servicio web, y las credenciales de acceso.</t>
+          <t>•  Si el link es el mismo para toda la flota, déjelo sólo en la primera fila y anótelo en la columna Notas.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>•  Cada cuánto reporta cada unidad (cada minuto, cada 5 minutos…).</t>
+          <t>•  Con ese link, la plataforma mostrará un acceso directo al seguimiento de cada unidad.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>•  Si no cuentan con GPS, el kilometraje y la posición los capturará a mano el Administrador de Unidad.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="5" t="inlineStr">
+          <t>•  El kilometraje semanal seguirá capturándose en el formulario del Administrador de Unidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>Assets y accesos</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>•  Logotipo en formato vectorial (SVG, AI o EPS). Si solo hay PNG: mínimo 1000 px de ancho y fondo transparente.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>•  De ser posible, tres variantes: a color, en negro y en blanco.</t>
+          <t>•  Logotipo en formato vectorial (SVG, AI o EPS). Si solo hay PNG: mínimo 1000 px de ancho y fondo transparente.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>•  Códigos de color institucionales en HEX y tipografía, si deben respetarse.</t>
+          <t>•  De ser posible, tres variantes: a color, en negro y en blanco.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>•  Códigos de color institucionales en HEX y tipografía, si deben respetarse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>•  Datos personales: teléfono, correo y licencia del conductor se tratan como datos personales; conviene que su aviso de privacidad los cubra.</t>
         </is>
@@ -948,7 +958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:X43"/>
+  <dimension ref="A1:Z43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -975,6 +985,8 @@
     <col width="14" customWidth="1" min="22" max="22"/>
     <col width="14" customWidth="1" min="23" max="23"/>
     <col width="34" customWidth="1" min="24" max="24"/>
+    <col width="42" customWidth="1" min="25" max="25"/>
+    <col width="30" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -998,6 +1010,11 @@
           <t>PÓLIZA DE SEGURO</t>
         </is>
       </c>
+      <c r="Y1" s="6" t="inlineStr">
+        <is>
+          <t>SEGUIMIENTO GPS</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
@@ -1120,6 +1137,16 @@
           <t>Cobertura</t>
         </is>
       </c>
+      <c r="Y2" s="7" t="inlineStr">
+        <is>
+          <t>Link de seguimiento (GPS)</t>
+        </is>
+      </c>
+      <c r="Z2" s="7" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
@@ -1230,6 +1257,12 @@
           <t>Cobertura amplia · RC $4,000,000</t>
         </is>
       </c>
+      <c r="Y3" s="8" t="inlineStr">
+        <is>
+          <t>https://seguimiento.proveedor.mx/u/ABC123</t>
+        </is>
+      </c>
+      <c r="Z3" s="8" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="9" t="n"/>
@@ -1256,6 +1289,8 @@
       <c r="V4" s="9" t="n"/>
       <c r="W4" s="9" t="n"/>
       <c r="X4" s="9" t="n"/>
+      <c r="Y4" s="9" t="n"/>
+      <c r="Z4" s="9" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="10" t="n"/>
@@ -1282,6 +1317,8 @@
       <c r="V5" s="10" t="n"/>
       <c r="W5" s="10" t="n"/>
       <c r="X5" s="10" t="n"/>
+      <c r="Y5" s="10" t="n"/>
+      <c r="Z5" s="10" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="n"/>
@@ -1308,6 +1345,8 @@
       <c r="V6" s="9" t="n"/>
       <c r="W6" s="9" t="n"/>
       <c r="X6" s="9" t="n"/>
+      <c r="Y6" s="9" t="n"/>
+      <c r="Z6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="n"/>
@@ -1334,6 +1373,8 @@
       <c r="V7" s="10" t="n"/>
       <c r="W7" s="10" t="n"/>
       <c r="X7" s="10" t="n"/>
+      <c r="Y7" s="10" t="n"/>
+      <c r="Z7" s="10" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="n"/>
@@ -1360,6 +1401,8 @@
       <c r="V8" s="9" t="n"/>
       <c r="W8" s="9" t="n"/>
       <c r="X8" s="9" t="n"/>
+      <c r="Y8" s="9" t="n"/>
+      <c r="Z8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="n"/>
@@ -1386,6 +1429,8 @@
       <c r="V9" s="10" t="n"/>
       <c r="W9" s="10" t="n"/>
       <c r="X9" s="10" t="n"/>
+      <c r="Y9" s="10" t="n"/>
+      <c r="Z9" s="10" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="n"/>
@@ -1412,6 +1457,8 @@
       <c r="V10" s="9" t="n"/>
       <c r="W10" s="9" t="n"/>
       <c r="X10" s="9" t="n"/>
+      <c r="Y10" s="9" t="n"/>
+      <c r="Z10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="n"/>
@@ -1438,6 +1485,8 @@
       <c r="V11" s="10" t="n"/>
       <c r="W11" s="10" t="n"/>
       <c r="X11" s="10" t="n"/>
+      <c r="Y11" s="10" t="n"/>
+      <c r="Z11" s="10" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n"/>
@@ -1464,6 +1513,8 @@
       <c r="V12" s="9" t="n"/>
       <c r="W12" s="9" t="n"/>
       <c r="X12" s="9" t="n"/>
+      <c r="Y12" s="9" t="n"/>
+      <c r="Z12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="n"/>
@@ -1490,6 +1541,8 @@
       <c r="V13" s="10" t="n"/>
       <c r="W13" s="10" t="n"/>
       <c r="X13" s="10" t="n"/>
+      <c r="Y13" s="10" t="n"/>
+      <c r="Z13" s="10" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="n"/>
@@ -1516,6 +1569,8 @@
       <c r="V14" s="9" t="n"/>
       <c r="W14" s="9" t="n"/>
       <c r="X14" s="9" t="n"/>
+      <c r="Y14" s="9" t="n"/>
+      <c r="Z14" s="9" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="n"/>
@@ -1542,6 +1597,8 @@
       <c r="V15" s="10" t="n"/>
       <c r="W15" s="10" t="n"/>
       <c r="X15" s="10" t="n"/>
+      <c r="Y15" s="10" t="n"/>
+      <c r="Z15" s="10" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="n"/>
@@ -1568,6 +1625,8 @@
       <c r="V16" s="9" t="n"/>
       <c r="W16" s="9" t="n"/>
       <c r="X16" s="9" t="n"/>
+      <c r="Y16" s="9" t="n"/>
+      <c r="Z16" s="9" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="n"/>
@@ -1594,6 +1653,8 @@
       <c r="V17" s="10" t="n"/>
       <c r="W17" s="10" t="n"/>
       <c r="X17" s="10" t="n"/>
+      <c r="Y17" s="10" t="n"/>
+      <c r="Z17" s="10" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="9" t="n"/>
@@ -1620,6 +1681,8 @@
       <c r="V18" s="9" t="n"/>
       <c r="W18" s="9" t="n"/>
       <c r="X18" s="9" t="n"/>
+      <c r="Y18" s="9" t="n"/>
+      <c r="Z18" s="9" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="10" t="n"/>
@@ -1646,6 +1709,8 @@
       <c r="V19" s="10" t="n"/>
       <c r="W19" s="10" t="n"/>
       <c r="X19" s="10" t="n"/>
+      <c r="Y19" s="10" t="n"/>
+      <c r="Z19" s="10" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="9" t="n"/>
@@ -1672,6 +1737,8 @@
       <c r="V20" s="9" t="n"/>
       <c r="W20" s="9" t="n"/>
       <c r="X20" s="9" t="n"/>
+      <c r="Y20" s="9" t="n"/>
+      <c r="Z20" s="9" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="10" t="n"/>
@@ -1698,6 +1765,8 @@
       <c r="V21" s="10" t="n"/>
       <c r="W21" s="10" t="n"/>
       <c r="X21" s="10" t="n"/>
+      <c r="Y21" s="10" t="n"/>
+      <c r="Z21" s="10" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="9" t="n"/>
@@ -1724,6 +1793,8 @@
       <c r="V22" s="9" t="n"/>
       <c r="W22" s="9" t="n"/>
       <c r="X22" s="9" t="n"/>
+      <c r="Y22" s="9" t="n"/>
+      <c r="Z22" s="9" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="10" t="n"/>
@@ -1750,6 +1821,8 @@
       <c r="V23" s="10" t="n"/>
       <c r="W23" s="10" t="n"/>
       <c r="X23" s="10" t="n"/>
+      <c r="Y23" s="10" t="n"/>
+      <c r="Z23" s="10" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="9" t="n"/>
@@ -1776,6 +1849,8 @@
       <c r="V24" s="9" t="n"/>
       <c r="W24" s="9" t="n"/>
       <c r="X24" s="9" t="n"/>
+      <c r="Y24" s="9" t="n"/>
+      <c r="Z24" s="9" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="10" t="n"/>
@@ -1802,6 +1877,8 @@
       <c r="V25" s="10" t="n"/>
       <c r="W25" s="10" t="n"/>
       <c r="X25" s="10" t="n"/>
+      <c r="Y25" s="10" t="n"/>
+      <c r="Z25" s="10" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="9" t="n"/>
@@ -1828,6 +1905,8 @@
       <c r="V26" s="9" t="n"/>
       <c r="W26" s="9" t="n"/>
       <c r="X26" s="9" t="n"/>
+      <c r="Y26" s="9" t="n"/>
+      <c r="Z26" s="9" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="10" t="n"/>
@@ -1854,6 +1933,8 @@
       <c r="V27" s="10" t="n"/>
       <c r="W27" s="10" t="n"/>
       <c r="X27" s="10" t="n"/>
+      <c r="Y27" s="10" t="n"/>
+      <c r="Z27" s="10" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="9" t="n"/>
@@ -1880,6 +1961,8 @@
       <c r="V28" s="9" t="n"/>
       <c r="W28" s="9" t="n"/>
       <c r="X28" s="9" t="n"/>
+      <c r="Y28" s="9" t="n"/>
+      <c r="Z28" s="9" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="10" t="n"/>
@@ -1906,6 +1989,8 @@
       <c r="V29" s="10" t="n"/>
       <c r="W29" s="10" t="n"/>
       <c r="X29" s="10" t="n"/>
+      <c r="Y29" s="10" t="n"/>
+      <c r="Z29" s="10" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="9" t="n"/>
@@ -1932,6 +2017,8 @@
       <c r="V30" s="9" t="n"/>
       <c r="W30" s="9" t="n"/>
       <c r="X30" s="9" t="n"/>
+      <c r="Y30" s="9" t="n"/>
+      <c r="Z30" s="9" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="10" t="n"/>
@@ -1958,6 +2045,8 @@
       <c r="V31" s="10" t="n"/>
       <c r="W31" s="10" t="n"/>
       <c r="X31" s="10" t="n"/>
+      <c r="Y31" s="10" t="n"/>
+      <c r="Z31" s="10" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="9" t="n"/>
@@ -1984,6 +2073,8 @@
       <c r="V32" s="9" t="n"/>
       <c r="W32" s="9" t="n"/>
       <c r="X32" s="9" t="n"/>
+      <c r="Y32" s="9" t="n"/>
+      <c r="Z32" s="9" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="10" t="n"/>
@@ -2010,6 +2101,8 @@
       <c r="V33" s="10" t="n"/>
       <c r="W33" s="10" t="n"/>
       <c r="X33" s="10" t="n"/>
+      <c r="Y33" s="10" t="n"/>
+      <c r="Z33" s="10" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="9" t="n"/>
@@ -2036,6 +2129,8 @@
       <c r="V34" s="9" t="n"/>
       <c r="W34" s="9" t="n"/>
       <c r="X34" s="9" t="n"/>
+      <c r="Y34" s="9" t="n"/>
+      <c r="Z34" s="9" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="10" t="n"/>
@@ -2062,6 +2157,8 @@
       <c r="V35" s="10" t="n"/>
       <c r="W35" s="10" t="n"/>
       <c r="X35" s="10" t="n"/>
+      <c r="Y35" s="10" t="n"/>
+      <c r="Z35" s="10" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="9" t="n"/>
@@ -2088,6 +2185,8 @@
       <c r="V36" s="9" t="n"/>
       <c r="W36" s="9" t="n"/>
       <c r="X36" s="9" t="n"/>
+      <c r="Y36" s="9" t="n"/>
+      <c r="Z36" s="9" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="10" t="n"/>
@@ -2114,6 +2213,8 @@
       <c r="V37" s="10" t="n"/>
       <c r="W37" s="10" t="n"/>
       <c r="X37" s="10" t="n"/>
+      <c r="Y37" s="10" t="n"/>
+      <c r="Z37" s="10" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="9" t="n"/>
@@ -2140,6 +2241,8 @@
       <c r="V38" s="9" t="n"/>
       <c r="W38" s="9" t="n"/>
       <c r="X38" s="9" t="n"/>
+      <c r="Y38" s="9" t="n"/>
+      <c r="Z38" s="9" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="10" t="n"/>
@@ -2166,6 +2269,8 @@
       <c r="V39" s="10" t="n"/>
       <c r="W39" s="10" t="n"/>
       <c r="X39" s="10" t="n"/>
+      <c r="Y39" s="10" t="n"/>
+      <c r="Z39" s="10" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="9" t="n"/>
@@ -2192,6 +2297,8 @@
       <c r="V40" s="9" t="n"/>
       <c r="W40" s="9" t="n"/>
       <c r="X40" s="9" t="n"/>
+      <c r="Y40" s="9" t="n"/>
+      <c r="Z40" s="9" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="10" t="n"/>
@@ -2218,6 +2325,8 @@
       <c r="V41" s="10" t="n"/>
       <c r="W41" s="10" t="n"/>
       <c r="X41" s="10" t="n"/>
+      <c r="Y41" s="10" t="n"/>
+      <c r="Z41" s="10" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="9" t="n"/>
@@ -2244,6 +2353,8 @@
       <c r="V42" s="9" t="n"/>
       <c r="W42" s="9" t="n"/>
       <c r="X42" s="9" t="n"/>
+      <c r="Y42" s="9" t="n"/>
+      <c r="Z42" s="9" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="10" t="n"/>
@@ -2270,13 +2381,16 @@
       <c r="V43" s="10" t="n"/>
       <c r="W43" s="10" t="n"/>
       <c r="X43" s="10" t="n"/>
+      <c r="Y43" s="10" t="n"/>
+      <c r="Z43" s="10" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="O1:S1"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="T1:X1"/>
+    <mergeCell ref="Y1:Z1"/>
     <mergeCell ref="J1:N1"/>
-    <mergeCell ref="O1:S1"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="J4:J43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no válido" error="Elija un estatus de la lista." type="list">

</xml_diff>